<commit_message>
Stage 8.20A.3: lock ranked trait effect contract
Stage 8.20A.3: lock ranked trait effect contract
</commit_message>
<xml_diff>
--- a/ContentSource/PlayerContent/FMCodex_Rules_Simplification_Draft.xlsx
+++ b/ContentSource/PlayerContent/FMCodex_Rules_Simplification_Draft.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="361">
   <si>
     <t>规则简化数据草稿</t>
   </si>
@@ -1000,6 +1000,132 @@
   </si>
   <si>
     <t>反越位专家旧等级</t>
+  </si>
+  <si>
+    <t>Direct</t>
+  </si>
+  <si>
+    <t>Shooting：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>无 DeadCorner 效果。</t>
+  </si>
+  <si>
+    <t>Control：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>不增加 Shooting；同一 Carrier 的平均公式不变。</t>
+  </si>
+  <si>
+    <t>Passing：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>两条实际路线共用同一 Trait。</t>
+  </si>
+  <si>
+    <t>Strength：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>仅实际高球接应。</t>
+  </si>
+  <si>
+    <t>Speed：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>不使用 Shooting 或 Control。</t>
+  </si>
+  <si>
+    <t>Feet / BehindDefense P1</t>
+  </si>
+  <si>
+    <t>仅普通属性 Formula，不延续至单刀。</t>
+  </si>
+  <si>
+    <t>BehindDefense P1</t>
+  </si>
+  <si>
+    <t>出界无 Formula；不延续至单刀。</t>
+  </si>
+  <si>
+    <t>不增加 Speed。</t>
+  </si>
+  <si>
+    <t>实际选中的 Runner</t>
+  </si>
+  <si>
+    <t>未选中的候选不贡献。</t>
+  </si>
+  <si>
+    <t>不增加 Speed；候选不贡献。</t>
+  </si>
+  <si>
+    <t>Shooting + Passing：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>两项各加同一 Bonus，再取 max。</t>
+  </si>
+  <si>
+    <t>不恢复 LS，不影响 Power。</t>
+  </si>
+  <si>
+    <t>两项各加同一 Bonus，再取 max；不影响 Panenka。</t>
+  </si>
+  <si>
+    <t>Marker</t>
+  </si>
+  <si>
+    <t>Defense：每项属性 S+3 / A+2 / B+1，先加成再用原系数。</t>
+  </si>
+  <si>
+    <t>仅实际防守 Formula 参与者。</t>
+  </si>
+  <si>
+    <t>不增加同一 Marker 的 Speed。</t>
+  </si>
+  <si>
+    <t>Marker 与 Helper 协防区分。</t>
+  </si>
+  <si>
+    <t>Helper</t>
+  </si>
+  <si>
+    <t>缺席 Helper 不贡献。</t>
+  </si>
+  <si>
+    <t>不改为 Defense；缺席不贡献。</t>
+  </si>
+  <si>
+    <t>无属性比较的路径不制造 Marker Formula。</t>
+  </si>
+  <si>
+    <t>不增加 Strength；缺席不贡献。</t>
+  </si>
+  <si>
+    <t>出界无 Formula；缺席不贡献。</t>
+  </si>
+  <si>
+    <t>实际选中的 Helper</t>
+  </si>
+  <si>
+    <t>非 GK；未选中的候选不贡献。</t>
+  </si>
+  <si>
+    <t>不增加 Speed；未选中的候选不贡献。</t>
+  </si>
+  <si>
+    <t>Trait taxonomy v1 · 24 项效果已锁定</t>
+  </si>
+  <si>
+    <t>Stage 8.20A.3：23 Ranked + 1 Binary 效果已批准，尚未实施。仅在本次实际 Formula 读取对应角色属性时应用 Ranked。</t>
+  </si>
+  <si>
+    <t>Ranked 统一 S+3 / A+2 / B+1；EffectiveAttribute = BaseAttribute + Bonus，再用原系数／max。基础值保留，不设最终值奖励。</t>
+  </si>
+  <si>
+    <t>不同实际参与者可同时生效。同一参与者在同一 Formula 至多匹配一个 Ranked，重复匹配是配置错误；不设优先级、递减或总上限。</t>
+  </si>
+  <si>
+    <t>Stage 8.20A.3 已锁定 23 Ranked：S+3 / A+2 / B+1，属性加成先于原系数；近任意球与点球两项同加再取 max。Binary 例外保留。全部尚未实施，详见 TraitCatalog。</t>
   </si>
 </sst>
 </file>
@@ -2011,7 +2137,7 @@
         <v>23</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>224</v>
+        <v>360</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="60" customHeight="1">
@@ -2043,7 +2169,7 @@
         <v>29</v>
       </c>
       <c r="B18" s="10" t="str">
-        <v>先审核 AutoFillReview 中的 Codex 分配及本阶段名单审查结论。修订与最终 Trait 效果由产品确认；不自动开始 runtime/canonical 迁移。</v>
+        <v>名单审查继续参照 AutoFillReview。Trait 效果已由 Stage 8.20A.3 锁定，名单平衡另行审核；不自动开始 runtime/canonical 迁移。</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="60" customHeight="1">
@@ -6611,7 +6737,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="26.1" customHeight="1">
       <c r="A1" s="18" t="s">
-        <v>237</v>
+        <v>356</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -6643,7 +6769,7 @@
     </row>
     <row r="3" spans="1:12" ht="26.1" customHeight="1">
       <c r="A3" s="15" t="s">
-        <v>239</v>
+        <v>357</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -6723,7 +6849,7 @@
         <v>248</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>249</v>
+        <v>319</v>
       </c>
       <c r="F6" s="21" t="s">
         <v>250</v>
@@ -6738,13 +6864,13 @@
         <v>253</v>
       </c>
       <c r="J6" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K6" s="21" t="s">
-        <v>199</v>
+        <v>320</v>
       </c>
       <c r="L6" s="21" t="s">
-        <v>254</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="48" customHeight="1">
@@ -6761,7 +6887,7 @@
         <v>256</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>249</v>
+        <v>319</v>
       </c>
       <c r="F7" s="21" t="s">
         <v>250</v>
@@ -6776,13 +6902,13 @@
         <v>253</v>
       </c>
       <c r="J7" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K7" s="21" t="s">
-        <v>199</v>
+        <v>322</v>
       </c>
       <c r="L7" s="21" t="s">
-        <v>254</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="48" customHeight="1">
@@ -6814,13 +6940,13 @@
         <v>253</v>
       </c>
       <c r="J8" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>199</v>
+        <v>324</v>
       </c>
       <c r="L8" s="21" t="s">
-        <v>260</v>
+        <v>325</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="48" customHeight="1">
@@ -6852,13 +6978,13 @@
         <v>253</v>
       </c>
       <c r="J9" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K9" s="21" t="s">
-        <v>199</v>
+        <v>326</v>
       </c>
       <c r="L9" s="21" t="s">
-        <v>254</v>
+        <v>327</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="48" customHeight="1">
@@ -6890,13 +7016,13 @@
         <v>253</v>
       </c>
       <c r="J10" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K10" s="21" t="s">
-        <v>199</v>
+        <v>328</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>254</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="48" customHeight="1">
@@ -6913,7 +7039,7 @@
         <v>267</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>249</v>
+        <v>330</v>
       </c>
       <c r="F11" s="21" t="s">
         <v>250</v>
@@ -6928,13 +7054,13 @@
         <v>253</v>
       </c>
       <c r="J11" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K11" s="21" t="s">
-        <v>199</v>
+        <v>324</v>
       </c>
       <c r="L11" s="21" t="s">
-        <v>254</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="96" customHeight="1">
@@ -6989,7 +7115,7 @@
         <v>267</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>276</v>
+        <v>332</v>
       </c>
       <c r="F13" s="21" t="s">
         <v>263</v>
@@ -7004,13 +7130,13 @@
         <v>253</v>
       </c>
       <c r="J13" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K13" s="21" t="s">
-        <v>199</v>
+        <v>328</v>
       </c>
       <c r="L13" s="21" t="s">
-        <v>254</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="48" customHeight="1">
@@ -7042,13 +7168,13 @@
         <v>253</v>
       </c>
       <c r="J14" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K14" s="21" t="s">
-        <v>199</v>
+        <v>322</v>
       </c>
       <c r="L14" s="21" t="s">
-        <v>254</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="48" customHeight="1">
@@ -7068,7 +7194,7 @@
         <v>262</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>281</v>
+        <v>335</v>
       </c>
       <c r="G15" s="21" t="s">
         <v>251</v>
@@ -7080,13 +7206,13 @@
         <v>253</v>
       </c>
       <c r="J15" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K15" s="21" t="s">
-        <v>199</v>
+        <v>326</v>
       </c>
       <c r="L15" s="21" t="s">
-        <v>282</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="48" customHeight="1">
@@ -7106,7 +7232,7 @@
         <v>265</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>281</v>
+        <v>335</v>
       </c>
       <c r="G16" s="21" t="s">
         <v>251</v>
@@ -7118,13 +7244,13 @@
         <v>253</v>
       </c>
       <c r="J16" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K16" s="21" t="s">
-        <v>199</v>
+        <v>322</v>
       </c>
       <c r="L16" s="21" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="48" customHeight="1">
@@ -7141,7 +7267,7 @@
         <v>285</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>286</v>
+        <v>319</v>
       </c>
       <c r="F17" s="21" t="s">
         <v>287</v>
@@ -7156,13 +7282,13 @@
         <v>253</v>
       </c>
       <c r="J17" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K17" s="21" t="s">
-        <v>199</v>
+        <v>338</v>
       </c>
       <c r="L17" s="21" t="s">
-        <v>254</v>
+        <v>339</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="48" customHeight="1">
@@ -7179,7 +7305,7 @@
         <v>289</v>
       </c>
       <c r="E18" s="21" t="s">
-        <v>286</v>
+        <v>319</v>
       </c>
       <c r="F18" s="21" t="s">
         <v>287</v>
@@ -7194,13 +7320,13 @@
         <v>253</v>
       </c>
       <c r="J18" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K18" s="21" t="s">
-        <v>199</v>
+        <v>320</v>
       </c>
       <c r="L18" s="21" t="s">
-        <v>254</v>
+        <v>340</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="48" customHeight="1">
@@ -7217,7 +7343,7 @@
         <v>291</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>286</v>
+        <v>319</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>287</v>
@@ -7232,13 +7358,13 @@
         <v>253</v>
       </c>
       <c r="J19" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K19" s="21" t="s">
-        <v>199</v>
+        <v>338</v>
       </c>
       <c r="L19" s="21" t="s">
-        <v>254</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="48" customHeight="1">
@@ -7255,10 +7381,10 @@
         <v>248</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
       <c r="F20" s="21" t="s">
-        <v>294</v>
+        <v>342</v>
       </c>
       <c r="G20" s="21" t="s">
         <v>251</v>
@@ -7270,13 +7396,13 @@
         <v>253</v>
       </c>
       <c r="J20" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K20" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L20" s="21" t="s">
-        <v>254</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" spans="1:12" ht="48" customHeight="1">
@@ -7293,10 +7419,10 @@
         <v>256</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>293</v>
+        <v>319</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>294</v>
+        <v>342</v>
       </c>
       <c r="G21" s="21" t="s">
         <v>251</v>
@@ -7308,13 +7434,13 @@
         <v>253</v>
       </c>
       <c r="J21" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K21" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L21" s="21" t="s">
-        <v>254</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="48" customHeight="1">
@@ -7334,7 +7460,7 @@
         <v>259</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>297</v>
+        <v>342</v>
       </c>
       <c r="G22" s="21" t="s">
         <v>251</v>
@@ -7346,13 +7472,13 @@
         <v>253</v>
       </c>
       <c r="J22" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K22" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L22" s="21" t="s">
-        <v>298</v>
+        <v>346</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="48" customHeight="1">
@@ -7372,7 +7498,7 @@
         <v>262</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="G23" s="21" t="s">
         <v>251</v>
@@ -7384,13 +7510,13 @@
         <v>253</v>
       </c>
       <c r="J23" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K23" s="21" t="s">
-        <v>199</v>
+        <v>326</v>
       </c>
       <c r="L23" s="21" t="s">
-        <v>254</v>
+        <v>348</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="48" customHeight="1">
@@ -7410,7 +7536,7 @@
         <v>265</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="G24" s="21" t="s">
         <v>251</v>
@@ -7422,13 +7548,13 @@
         <v>253</v>
       </c>
       <c r="J24" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K24" s="21" t="s">
-        <v>199</v>
+        <v>328</v>
       </c>
       <c r="L24" s="21" t="s">
-        <v>254</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" spans="1:12" ht="48" customHeight="1">
@@ -7445,10 +7571,10 @@
         <v>267</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>303</v>
+        <v>330</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="G25" s="21" t="s">
         <v>251</v>
@@ -7460,13 +7586,13 @@
         <v>253</v>
       </c>
       <c r="J25" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K25" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L25" s="21" t="s">
-        <v>254</v>
+        <v>350</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="48" customHeight="1">
@@ -7486,7 +7612,7 @@
         <v>278</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="G26" s="21" t="s">
         <v>251</v>
@@ -7498,13 +7624,13 @@
         <v>253</v>
       </c>
       <c r="J26" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K26" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L26" s="21" t="s">
-        <v>254</v>
+        <v>351</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="48" customHeight="1">
@@ -7521,10 +7647,10 @@
         <v>267</v>
       </c>
       <c r="E27" s="21" t="s">
-        <v>276</v>
+        <v>332</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>300</v>
+        <v>347</v>
       </c>
       <c r="G27" s="21" t="s">
         <v>251</v>
@@ -7536,13 +7662,13 @@
         <v>253</v>
       </c>
       <c r="J27" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K27" s="21" t="s">
-        <v>199</v>
+        <v>328</v>
       </c>
       <c r="L27" s="21" t="s">
-        <v>254</v>
+        <v>352</v>
       </c>
     </row>
     <row r="28" spans="1:12" ht="48" customHeight="1">
@@ -7562,7 +7688,7 @@
         <v>262</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>308</v>
+        <v>353</v>
       </c>
       <c r="G28" s="21" t="s">
         <v>251</v>
@@ -7574,13 +7700,13 @@
         <v>253</v>
       </c>
       <c r="J28" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K28" s="21" t="s">
-        <v>199</v>
+        <v>326</v>
       </c>
       <c r="L28" s="21" t="s">
-        <v>282</v>
+        <v>354</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="48" customHeight="1">
@@ -7600,7 +7726,7 @@
         <v>265</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>308</v>
+        <v>353</v>
       </c>
       <c r="G29" s="21" t="s">
         <v>251</v>
@@ -7612,13 +7738,13 @@
         <v>253</v>
       </c>
       <c r="J29" s="21" t="s">
-        <v>199</v>
+        <v>272</v>
       </c>
       <c r="K29" s="21" t="s">
-        <v>199</v>
+        <v>343</v>
       </c>
       <c r="L29" s="21" t="s">
-        <v>282</v>
+        <v>355</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="26.1" customHeight="1">
@@ -7701,7 +7827,7 @@
     </row>
     <row r="35" spans="1:12" ht="26.1" customHeight="1">
       <c r="A35" s="15" t="s">
-        <v>313</v>
+        <v>358</v>
       </c>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
@@ -7733,7 +7859,7 @@
     </row>
     <row r="37" spans="1:12" ht="26.1" customHeight="1">
       <c r="A37" s="15" t="s">
-        <v>315</v>
+        <v>359</v>
       </c>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>

</xml_diff>